<commit_message>
Migrated Home contacts and organization to product.
</commit_message>
<xml_diff>
--- a/src/main/resources/Field_Values.xlsx
+++ b/src/main/resources/Field_Values.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22730"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6CA980A-EB27-45BF-AB7A-72D4083AA088}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E95EF059-0F77-4F73-BCEC-6F40BE1EF085}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="16" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ContactCreation" sheetId="1" r:id="rId1"/>
@@ -132,9 +132,6 @@
     <t>fieldBudget_Categories__c</t>
   </si>
   <si>
-    <t>PERSONNEL</t>
-  </si>
-  <si>
     <t>fieldIndirectCostRateType__c</t>
   </si>
   <si>
@@ -613,13 +610,16 @@
   </si>
   <si>
     <t>fieldEstimatedFTEToBeHired__c</t>
+  </si>
+  <si>
+    <t>Personnel</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -720,6 +720,18 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF222222"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -748,7 +760,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -827,6 +839,11 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1110,14 +1127,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.21875" customWidth="1"/>
-    <col min="3" max="3" width="31.5546875" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.19921875" customWidth="1"/>
+    <col min="3" max="3" width="31.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1128,7 +1145,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1139,7 +1156,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1150,7 +1167,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1161,7 +1178,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1184,13 +1201,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAD7FB55-E8AD-485D-A372-6318A9353130}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="18.88671875" customWidth="1"/>
-    <col min="3" max="3" width="31.44140625" customWidth="1"/>
+    <col min="2" max="2" width="18.86328125" customWidth="1"/>
+    <col min="3" max="3" width="31.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1201,7 +1218,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1209,10 +1226,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1220,10 +1237,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1231,10 +1248,10 @@
         <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1242,10 +1259,10 @@
         <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1256,18 +1273,18 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1275,10 +1292,10 @@
         <v>18</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -1301,14 +1318,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E3D1CB4-74AD-4C7B-86A6-6D8597EFB79A}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="43.77734375" customWidth="1"/>
+    <col min="3" max="3" width="43.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1319,7 +1336,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1327,10 +1344,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="50.4" x14ac:dyDescent="0.3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="49.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1338,10 +1355,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1349,10 +1366,10 @@
         <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1360,10 +1377,10 @@
         <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1374,15 +1391,15 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>45</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1396,14 +1413,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D415097A-F360-43DD-83BE-32D88672EF13}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.21875" customWidth="1"/>
-    <col min="3" max="3" width="28.21875" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.19921875" customWidth="1"/>
+    <col min="3" max="3" width="28.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1414,7 +1431,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1422,10 +1439,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1433,10 +1450,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1444,10 +1461,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1470,14 +1487,14 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C84DBADC-4CFE-43C9-B33B-FB1978F25849}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.77734375" customWidth="1"/>
-    <col min="3" max="3" width="26.88671875" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.796875" customWidth="1"/>
+    <col min="3" max="3" width="26.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1488,7 +1505,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1499,7 +1516,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1510,7 +1527,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1518,10 +1535,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1532,15 +1549,15 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1555,13 +1572,13 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{410A8461-2BAC-4994-A5A0-900D2EAF4F3E}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="24.109375" customWidth="1"/>
-    <col min="3" max="3" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.1328125" customWidth="1"/>
+    <col min="3" max="3" width="22.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1572,7 +1589,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1583,7 +1600,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1594,7 +1611,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1616,13 +1633,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAFCF55F-195A-445C-9058-59993E2BC9ED}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="27.44140625" customWidth="1"/>
-    <col min="3" max="3" width="26.21875" customWidth="1"/>
+    <col min="2" max="2" width="27.46484375" customWidth="1"/>
+    <col min="3" max="3" width="26.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1633,7 +1650,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1644,7 +1661,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1655,7 +1672,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1666,7 +1683,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1677,7 +1694,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1688,7 +1705,7 @@
         <v>12345678</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1710,14 +1727,14 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDD507A7-A1D7-4C66-91DC-C17845AA6092}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="255.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="255.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1728,7 +1745,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1739,7 +1756,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1750,7 +1767,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1761,7 +1778,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1772,7 +1789,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1783,7 +1800,7 @@
         <v>12345678</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1794,7 +1811,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1817,14 +1834,14 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25B9AAB7-BC0B-48A4-8063-5D4A8BC952DC}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" customWidth="1"/>
-    <col min="2" max="2" width="26.5546875" customWidth="1"/>
-    <col min="3" max="3" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.46484375" customWidth="1"/>
+    <col min="2" max="2" width="26.53125" customWidth="1"/>
+    <col min="3" max="3" width="40.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
@@ -1835,70 +1852,70 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A2" s="28" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A3" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="29" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="30" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A3" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="29" t="s">
-        <v>50</v>
-      </c>
       <c r="C3" s="31" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A4" s="28" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="29" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C4" s="29">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="28" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="32" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A6" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="29" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A6" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="29" t="s">
+      <c r="C6" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="32" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" s="28" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" s="27" t="s">
         <v>57</v>
-      </c>
-      <c r="C7" s="27" t="s">
-        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1910,14 +1927,14 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D57C0A7E-0484-41B3-98B5-765D1318644D}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="19.109375" customWidth="1"/>
-    <col min="2" max="2" width="26.77734375" customWidth="1"/>
+    <col min="1" max="1" width="19.1328125" customWidth="1"/>
+    <col min="2" max="2" width="26.796875" customWidth="1"/>
     <col min="3" max="3" width="42.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1928,37 +1945,37 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="9" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>61</v>
-      </c>
       <c r="C3" s="1" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -1969,14 +1986,14 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90D837CB-E465-4E28-A130-5D8C398A0EED}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="13.6640625" customWidth="1"/>
-    <col min="2" max="2" width="36.5546875" customWidth="1"/>
-    <col min="3" max="3" width="57.88671875" customWidth="1"/>
+    <col min="2" max="2" width="36.53125" customWidth="1"/>
+    <col min="3" max="3" width="57.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1987,59 +2004,59 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="17" t="s">
+    </row>
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="16" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="16" t="s">
+      <c r="C4" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="C4" s="17" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="16" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="16" t="s">
+      <c r="C5" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="C5" s="15" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="16" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="16" t="s">
+      <c r="C6" s="15" t="s">
         <v>69</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -2050,14 +2067,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07A8DFDE-CC9C-46BE-84ED-CACACDED0505}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5546875" customWidth="1"/>
+    <col min="3" max="3" width="23.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2068,7 +2085,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2079,7 +2096,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -2090,7 +2107,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -2112,14 +2129,14 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AE13280-37FF-469C-B491-B5A066179CFD}">
   <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" customWidth="1"/>
+    <col min="1" max="1" width="12.53125" customWidth="1"/>
     <col min="2" max="2" width="41.6640625" customWidth="1"/>
-    <col min="3" max="3" width="52.5546875" customWidth="1"/>
+    <col min="3" max="3" width="52.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
@@ -2130,320 +2147,320 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="36" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B2" s="36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C2" s="34">
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="34" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B3" s="36" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C3" s="34">
         <v>199</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="B4" s="36" t="s">
-        <v>73</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="34" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" s="36" t="s">
-        <v>75</v>
-      </c>
-      <c r="C5" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="34" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" s="36" t="s">
+      <c r="C7" s="34" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="C6" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="34" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7" s="34" t="s">
+      <c r="B9" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="34" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="34" t="s">
-        <v>56</v>
-      </c>
-      <c r="B8" s="34" t="s">
-        <v>87</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B9" s="34" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="C9" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B10" s="34" t="s">
+      <c r="C10" s="34" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="C10" s="34" t="s">
+      <c r="C11" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A13" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A14" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" s="34" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B11" s="34" t="s">
-        <v>80</v>
-      </c>
-      <c r="C11" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B12" s="34" t="s">
-        <v>81</v>
-      </c>
-      <c r="C12" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B13" s="34" t="s">
+      <c r="C14" s="34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A15" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B15" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="C13" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B14" s="34" t="s">
-        <v>181</v>
-      </c>
-      <c r="C14" s="34">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B15" s="34" t="s">
+      <c r="C15" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A16" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="C15" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B16" s="34" t="s">
+      <c r="C16" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A17" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B17" s="34" t="s">
         <v>84</v>
-      </c>
-      <c r="C16" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B17" s="34" t="s">
-        <v>85</v>
       </c>
       <c r="C17" s="34">
         <v>50000</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" s="34" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B18" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A19" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="C18" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B19" s="34" t="s">
+      <c r="C19" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A20" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B20" s="34" t="s">
+      <c r="C20" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A21" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" s="34" t="s">
         <v>88</v>
       </c>
-      <c r="C20" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B21" s="34" t="s">
+      <c r="C21" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A22" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="C21" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B22" s="34" t="s">
+      <c r="C22" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A23" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="C22" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B23" s="34" t="s">
+      <c r="C23" s="34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A24" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B24" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="C23" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B24" s="34" t="s">
+      <c r="C24" s="34" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A25" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="C24" s="34" t="s">
+      <c r="C25" s="34" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B25" s="34" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A26" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" s="34" t="s">
         <v>93</v>
       </c>
-      <c r="C25" s="34" t="s">
+      <c r="C26" s="34" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B26" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="C26" s="34" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A27" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B27" s="34" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B27" s="34" t="s">
+      <c r="C27" s="34" t="s">
         <v>185</v>
       </c>
-      <c r="C27" s="34" t="s">
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A28" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B28" s="35" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B28" s="35" t="s">
+      <c r="C28" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="C28" s="34" t="s">
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A29" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B29" s="34" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B29" s="34" t="s">
+      <c r="C29" s="34" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A30" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B30" s="34" t="s">
         <v>189</v>
-      </c>
-      <c r="C29" s="34" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B30" s="34" t="s">
-        <v>190</v>
       </c>
       <c r="C30" s="33">
         <v>2</v>
@@ -2458,14 +2475,14 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C9D7AD-DD13-4E10-B333-6FC741B3BFBF}">
   <dimension ref="A1:C31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="11.109375" customWidth="1"/>
-    <col min="2" max="2" width="39.5546875" customWidth="1"/>
+    <col min="1" max="1" width="11.1328125" customWidth="1"/>
+    <col min="2" max="2" width="39.53125" customWidth="1"/>
     <col min="3" max="3" width="40.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -2476,334 +2493,334 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="19" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C2" s="21">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="19" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C4" s="21" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C4" s="21" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="20" t="s">
+      <c r="C5" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="C5" s="21" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="21" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" s="21" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="23" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="23" t="s">
+      <c r="C7" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="C7" s="21" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="23" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="23" t="s">
+      <c r="C8" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="C8" s="21" t="s">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="23" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="23" t="s">
+      <c r="C9" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="C9" s="21" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="23" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="23" t="s">
+      <c r="C10" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="C10" s="21" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="23" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="23" t="s">
+      <c r="C11" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="C11" s="21" t="s">
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="23" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" s="23" t="s">
+      <c r="C12" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="C12" s="21" t="s">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A13" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="23" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="23" t="s">
+      <c r="C13" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="C13" s="21" t="s">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A14" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="23" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" s="23" t="s">
+      <c r="C14" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="C14" s="21" t="s">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A15" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="23" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15" s="23" t="s">
+      <c r="C15" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="C15" s="21" t="s">
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A16" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="23" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B16" s="23" t="s">
+      <c r="C16" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="C16" s="21" t="s">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A17" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="23" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B17" s="23" t="s">
+      <c r="C17" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="C17" s="21" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A18" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="23" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B18" s="23" t="s">
+      <c r="C18" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="C18" s="21" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A19" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="23" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B19" s="23" t="s">
+      <c r="C19" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="C19" s="21" t="s">
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A20" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="23" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B20" s="23" t="s">
+      <c r="C20" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="C20" s="21" t="s">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A21" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="23" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B21" s="23" t="s">
+      <c r="C21" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="C21" s="21" t="s">
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A22" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="23" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B22" s="23" t="s">
+      <c r="C22" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="C22" s="21" t="s">
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A23" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="23" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B23" s="23" t="s">
+      <c r="C23" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="C23" s="21" t="s">
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A24" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" s="23" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B24" s="23" t="s">
+      <c r="C24" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="C24" s="21" t="s">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A25" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="23" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B25" s="23" t="s">
+      <c r="C25" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="C25" s="21" t="s">
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A26" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" s="23" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B26" s="23" t="s">
+      <c r="C26" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="C26" s="21" t="s">
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A27" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27" s="23" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B27" s="23" t="s">
+      <c r="C27" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="C27" s="21" t="s">
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A28" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" s="23" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B28" s="23" t="s">
+      <c r="C28" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="C28" s="21" t="s">
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A29" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="23" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B29" s="23" t="s">
+      <c r="C29" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="C29" s="21" t="s">
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A30" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B30" s="23" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B30" s="23" t="s">
+      <c r="C30" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="C30" s="21" t="s">
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A31" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" s="23" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="23" t="s">
+      <c r="C31" s="21" t="s">
         <v>148</v>
-      </c>
-      <c r="C31" s="21" t="s">
-        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -2814,14 +2831,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C825052-5BFB-48CE-AF18-A05985C2E861}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" customWidth="1"/>
-    <col min="3" max="3" width="26.21875" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.46484375" customWidth="1"/>
+    <col min="3" max="3" width="26.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2832,7 +2849,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2843,7 +2860,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -2854,7 +2871,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -2865,7 +2882,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2876,7 +2893,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -2887,7 +2904,7 @@
         <v>12345678</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -2909,14 +2926,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C54FC4-ECE0-4935-82B1-FA8D76408EA8}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="2" width="23.44140625" customWidth="1"/>
-    <col min="3" max="3" width="30.88671875" customWidth="1"/>
+    <col min="1" max="1" width="14.796875" customWidth="1"/>
+    <col min="2" max="2" width="23.46484375" customWidth="1"/>
+    <col min="3" max="3" width="30.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2927,7 +2944,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2938,7 +2955,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -2949,7 +2966,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -2960,7 +2977,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2971,7 +2988,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -2982,7 +2999,7 @@
         <v>12345678</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -2993,7 +3010,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -3015,14 +3032,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E468D78-1254-4AD2-810C-41AE4E131ED6}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" customWidth="1"/>
-    <col min="2" max="2" width="25.5546875" customWidth="1"/>
+    <col min="1" max="1" width="18.46484375" customWidth="1"/>
+    <col min="2" max="2" width="25.53125" customWidth="1"/>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3033,7 +3050,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -3041,10 +3058,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -3052,10 +3069,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -3066,7 +3083,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -3077,7 +3094,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -3088,7 +3105,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -3099,7 +3116,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -3110,7 +3127,7 @@
         <v>41102</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -3118,29 +3135,29 @@
         <v>18</v>
       </c>
       <c r="C9" s="24" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="C10" s="24" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="12" t="s">
+    <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C11" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="C11" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -3155,87 +3172,87 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3165D747-C28E-4C3E-96DA-2777CB00933A}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="25.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="37" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="3" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="37" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="3" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="5">
-        <v>-10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="s">
+      <c r="C3" s="39">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="38" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="38" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="38" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C6" s="39">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C7" s="39">
         <v>365</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -3247,13 +3264,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE2AE6E5-9BA0-4079-BFA8-85F960DC3870}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="25.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3264,70 +3281,70 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="3" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="37" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="3" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="5">
-        <v>-10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="s">
+      <c r="C3" s="39">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="38" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="38" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="38" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C6" s="39">
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C7" s="39">
         <v>365</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -3338,13 +3355,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB063D14-2E1A-4894-A22D-BD2B91269468}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="25.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.19921875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3355,7 +3372,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3363,84 +3380,84 @@
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="s">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C5" s="7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="s">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>36</v>
       </c>
       <c r="C6" s="8">
         <v>20301</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A9" t="s">
         <v>3</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -3455,14 +3472,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A2F5532-64E8-4157-849F-E59312F5A712}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="44.21875" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" customWidth="1"/>
+    <col min="2" max="2" width="44.19921875" customWidth="1"/>
+    <col min="3" max="3" width="20.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
@@ -3473,125 +3490,125 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C2">
         <v>456123789</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B3" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="C3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" t="s">
         <v>154</v>
       </c>
-      <c r="C3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" t="s">
         <v>155</v>
       </c>
-      <c r="C4" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" t="s">
         <v>156</v>
       </c>
-      <c r="C5" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>163</v>
+      </c>
+      <c r="B7" t="s">
         <v>157</v>
       </c>
-      <c r="C6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>164</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>163</v>
+      </c>
+      <c r="B8" t="s">
         <v>158</v>
       </c>
-      <c r="C7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>164</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>163</v>
+      </c>
+      <c r="B9" t="s">
         <v>159</v>
       </c>
-      <c r="C8" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>164</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>163</v>
+      </c>
+      <c r="B10" t="s">
         <v>160</v>
       </c>
-      <c r="C9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>164</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B11" t="s">
         <v>161</v>
       </c>
-      <c r="C10" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>164</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>163</v>
+      </c>
+      <c r="B12" t="s">
         <v>162</v>
       </c>
-      <c r="C11" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>164</v>
-      </c>
-      <c r="B12" t="s">
-        <v>163</v>
-      </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Application and Pre-Application modules
</commit_message>
<xml_diff>
--- a/src/main/resources/Field_Values.xlsx
+++ b/src/main/resources/Field_Values.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22827"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDE26178-2DAB-411E-A150-D5E91743C44E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E681FD-7FD9-426A-8CE6-7BE9E951B5BE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="13" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="16" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ContactCreation" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="189">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -183,9 +183,6 @@
     <t>automationExternalNonFederalContact@yopmail.com</t>
   </si>
   <si>
-    <t>Health State Organization</t>
-  </si>
-  <si>
     <t>fieldFederalAgency__c</t>
   </si>
   <si>
@@ -264,362 +261,359 @@
     <t>Non-Construction</t>
   </si>
   <si>
-    <t>fieldPreApplicationNeeded__c</t>
+    <t>Evaluation</t>
+  </si>
+  <si>
+    <t>fieldHaveWeReceivedAwardFromProgram__c</t>
+  </si>
+  <si>
+    <t>fieldJustificationofOurStandingAgency__c</t>
+  </si>
+  <si>
+    <t>fieldBusinessandTechnicaldomainKnowledge__c</t>
+  </si>
+  <si>
+    <t>fieldSkillSets__c</t>
+  </si>
+  <si>
+    <t>fieldNecessarySystemsAndFinancialTools__c</t>
+  </si>
+  <si>
+    <t>fieldQualifiedByOtherAgencies__c</t>
+  </si>
+  <si>
+    <t>fieldCollaborationandWorkShare__c</t>
+  </si>
+  <si>
+    <t>fieldMaintenanceEffortRequire__c</t>
+  </si>
+  <si>
+    <t>fieldIsProgramIncomeAnticipated__c</t>
+  </si>
+  <si>
+    <t>fieldRequiredPassThroughToSubrecipients__c</t>
+  </si>
+  <si>
+    <t>fieldLimitOnAdministrativeRate__c</t>
+  </si>
+  <si>
+    <t>fieldProgramSustainability__c</t>
+  </si>
+  <si>
+    <t>fieldLegalRequirementOrOtherCertification__c</t>
+  </si>
+  <si>
+    <t>fieldRichTextArea1__c</t>
+  </si>
+  <si>
+    <t>NFPG-Test3</t>
+  </si>
+  <si>
+    <t>Test Org 6</t>
+  </si>
+  <si>
+    <t>fieldApplicantEligibility__c</t>
+  </si>
+  <si>
+    <t>appEligibility</t>
+  </si>
+  <si>
+    <t>objectives</t>
+  </si>
+  <si>
+    <t>fieldAssistanceType__c</t>
+  </si>
+  <si>
+    <t>typesofassistance</t>
+  </si>
+  <si>
+    <t>fieldUsesAndUseRestrictions__c</t>
+  </si>
+  <si>
+    <t>users and user rest</t>
+  </si>
+  <si>
+    <t>fieldCredentialsDocumentation__c</t>
+  </si>
+  <si>
+    <t>credentials</t>
+  </si>
+  <si>
+    <t>fieldBeneficiaryEligibility__c</t>
+  </si>
+  <si>
+    <t>benificiary</t>
+  </si>
+  <si>
+    <t>fieldPreapplicationCoordination__c</t>
+  </si>
+  <si>
+    <t>preapplication</t>
+  </si>
+  <si>
+    <t>fieldApplicationProcedures__c</t>
+  </si>
+  <si>
+    <t>app procedures</t>
+  </si>
+  <si>
+    <t>fieldAwardProcedure__c</t>
+  </si>
+  <si>
+    <t>award procedure</t>
+  </si>
+  <si>
+    <t>fieldDeadlines__c</t>
+  </si>
+  <si>
+    <t>deadlines</t>
+  </si>
+  <si>
+    <t>fieldRangeofApprovalDisApprovalTime__c</t>
+  </si>
+  <si>
+    <t>range of approval</t>
+  </si>
+  <si>
+    <t>fieldAppeals__c</t>
+  </si>
+  <si>
+    <t>appeals</t>
+  </si>
+  <si>
+    <t>fieldRenewals__c</t>
+  </si>
+  <si>
+    <t>renewals</t>
+  </si>
+  <si>
+    <t>fieldCriteriaforSelectingProposals__c</t>
+  </si>
+  <si>
+    <t>criteria</t>
+  </si>
+  <si>
+    <t>fieldFormulaandMatchingRequirements__c</t>
+  </si>
+  <si>
+    <t>formula</t>
+  </si>
+  <si>
+    <t>fieldLengthandTimePhasingofAssistance__c</t>
+  </si>
+  <si>
+    <t>lengthandtime</t>
+  </si>
+  <si>
+    <t>fieldReports__c</t>
+  </si>
+  <si>
+    <t>reports</t>
+  </si>
+  <si>
+    <t>fieldAudits__c</t>
+  </si>
+  <si>
+    <t>audits</t>
+  </si>
+  <si>
+    <t>fieldRecords__c</t>
+  </si>
+  <si>
+    <t>records</t>
+  </si>
+  <si>
+    <t>fieldRegulationsGuidelinesAndLiterature__c</t>
+  </si>
+  <si>
+    <t>regulations</t>
+  </si>
+  <si>
+    <t>fieldAccountIdentification__c</t>
+  </si>
+  <si>
+    <t>accIdentification</t>
+  </si>
+  <si>
+    <t>fieldObligations__c</t>
+  </si>
+  <si>
+    <t>obligations</t>
+  </si>
+  <si>
+    <t>fieldRangeandAverageofFinancialAssistanc__c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">range </t>
+  </si>
+  <si>
+    <t>fieldProgramAccomplishments__c</t>
+  </si>
+  <si>
+    <t>accomplishments</t>
+  </si>
+  <si>
+    <t>fieldRegionalOrLocalOffice__c</t>
+  </si>
+  <si>
+    <t>rehional</t>
+  </si>
+  <si>
+    <t>fieldHeadquartersOffice__c</t>
+  </si>
+  <si>
+    <t>headq</t>
+  </si>
+  <si>
+    <t>fieldWebsiteAddress__c</t>
+  </si>
+  <si>
+    <t>website</t>
+  </si>
+  <si>
+    <t>fieldMailingCity</t>
+  </si>
+  <si>
+    <t>fieldMailingState</t>
+  </si>
+  <si>
+    <t>fieldNonFederalOrgamizationType__c</t>
+  </si>
+  <si>
+    <t>fieldDUNS__c</t>
+  </si>
+  <si>
+    <t>fieldAuthorizedOrganizationContact__c</t>
+  </si>
+  <si>
+    <t>fieldProjectAbstract__c</t>
+  </si>
+  <si>
+    <t>fieldLocation__c</t>
+  </si>
+  <si>
+    <t>fieldSupplementalFundsRequest__c</t>
+  </si>
+  <si>
+    <t>fieldAre_any_state_specific_forms_attached__c</t>
+  </si>
+  <si>
+    <t>fieldAre_space_requirements_met__c</t>
+  </si>
+  <si>
+    <t>fieldIT_requirements_met__c</t>
+  </si>
+  <si>
+    <t>fieldTraining_Requirements_Met__c</t>
+  </si>
+  <si>
+    <t>fieldAre_special_award_conditions_addressed__c</t>
+  </si>
+  <si>
+    <t>fieldAddition_pending_requirements__c</t>
+  </si>
+  <si>
+    <t>Checklist</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Project Abstract Value</t>
+  </si>
+  <si>
+    <t>Automation PM</t>
+  </si>
+  <si>
+    <t>Automation Runtime Contact</t>
+  </si>
+  <si>
+    <t>Automation External Federal Contact</t>
+  </si>
+  <si>
+    <t>Contact</t>
+  </si>
+  <si>
+    <t>Automation Runtime FederalContactsLengthCheck</t>
+  </si>
+  <si>
+    <t>AutomationExernalContactToCheckMaximum0123AutomationExernalContactToCheckMaximum0123</t>
+  </si>
+  <si>
+    <t>Test Address</t>
+  </si>
+  <si>
+    <t>Automation Runtime NF Program</t>
+  </si>
+  <si>
+    <t>Automation Runtime Internal Program</t>
+  </si>
+  <si>
+    <t>Automation Runtime NF Organization</t>
+  </si>
+  <si>
+    <t>Automation Internal Org</t>
+  </si>
+  <si>
+    <t>Automation Runtime Lead</t>
+  </si>
+  <si>
+    <t>aaaaaaaaa</t>
+  </si>
+  <si>
+    <t>fieldLevelofEffort__c</t>
+  </si>
+  <si>
+    <t>aaaaaa</t>
+  </si>
+  <si>
+    <t>aaaaaaa</t>
+  </si>
+  <si>
+    <t>sssssss</t>
+  </si>
+  <si>
+    <t>fieldDetailTechnicalKnowledge__c</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>fieldExplainRequiredResources__c</t>
+  </si>
+  <si>
+    <t>tst</t>
+  </si>
+  <si>
+    <t>fieldExplainRequiredRequirements__c</t>
+  </si>
+  <si>
+    <t>fieldEstimatedFTEToBeHired__c</t>
+  </si>
+  <si>
+    <t>Personnel</t>
+  </si>
+  <si>
+    <t>Automation External Federal Contact Test</t>
+  </si>
+  <si>
+    <t>Automation External Non Federal Contact Test</t>
+  </si>
+  <si>
+    <t>Department of Health</t>
   </si>
   <si>
     <t>fieldLetterOfIntentRequired__c</t>
   </si>
   <si>
-    <t>Evaluation</t>
-  </si>
-  <si>
-    <t>fieldHaveWeReceivedAwardFromProgram__c</t>
-  </si>
-  <si>
-    <t>fieldJustificationofOurStandingAgency__c</t>
-  </si>
-  <si>
-    <t>fieldBusinessandTechnicaldomainKnowledge__c</t>
-  </si>
-  <si>
-    <t>fieldSkillSets__c</t>
-  </si>
-  <si>
-    <t>fieldNecessarySystemsAndFinancialTools__c</t>
-  </si>
-  <si>
-    <t>fieldQualifiedByOtherAgencies__c</t>
-  </si>
-  <si>
-    <t>fieldCollaborationandWorkShare__c</t>
-  </si>
-  <si>
-    <t>fieldExpectedTotalAwardAmount__c</t>
-  </si>
-  <si>
-    <t>fieldMaintenanceEffortRequire__c</t>
-  </si>
-  <si>
-    <t>fieldIsProgramIncomeAnticipated__c</t>
-  </si>
-  <si>
-    <t>fieldIsMatchRequired__c</t>
-  </si>
-  <si>
-    <t>fieldRequiredPassThroughToSubrecipients__c</t>
-  </si>
-  <si>
-    <t>fieldDoesGrantAllowIndirect__c</t>
-  </si>
-  <si>
-    <t>fieldLimitOnAdministrativeRate__c</t>
-  </si>
-  <si>
-    <t>fieldProgramSustainability__c</t>
-  </si>
-  <si>
-    <t>fieldLegalRequirementOrOtherCertification__c</t>
-  </si>
-  <si>
-    <t>fieldRichTextArea1__c</t>
-  </si>
-  <si>
-    <t>NFPG-Test3</t>
-  </si>
-  <si>
-    <t>Test Org 6</t>
-  </si>
-  <si>
-    <t>fieldApplicantEligibility__c</t>
-  </si>
-  <si>
-    <t>appEligibility</t>
-  </si>
-  <si>
-    <t>objectives</t>
-  </si>
-  <si>
-    <t>fieldAssistanceType__c</t>
-  </si>
-  <si>
-    <t>typesofassistance</t>
-  </si>
-  <si>
-    <t>fieldUsesAndUseRestrictions__c</t>
-  </si>
-  <si>
-    <t>users and user rest</t>
-  </si>
-  <si>
-    <t>fieldCredentialsDocumentation__c</t>
-  </si>
-  <si>
-    <t>credentials</t>
-  </si>
-  <si>
-    <t>fieldBeneficiaryEligibility__c</t>
-  </si>
-  <si>
-    <t>benificiary</t>
-  </si>
-  <si>
-    <t>fieldPreapplicationCoordination__c</t>
-  </si>
-  <si>
-    <t>preapplication</t>
-  </si>
-  <si>
-    <t>fieldApplicationProcedures__c</t>
-  </si>
-  <si>
-    <t>app procedures</t>
-  </si>
-  <si>
-    <t>fieldAwardProcedure__c</t>
-  </si>
-  <si>
-    <t>award procedure</t>
-  </si>
-  <si>
-    <t>fieldDeadlines__c</t>
-  </si>
-  <si>
-    <t>deadlines</t>
-  </si>
-  <si>
-    <t>fieldRangeofApprovalDisApprovalTime__c</t>
-  </si>
-  <si>
-    <t>range of approval</t>
-  </si>
-  <si>
-    <t>fieldAppeals__c</t>
-  </si>
-  <si>
-    <t>appeals</t>
-  </si>
-  <si>
-    <t>fieldRenewals__c</t>
-  </si>
-  <si>
-    <t>renewals</t>
-  </si>
-  <si>
-    <t>fieldCriteriaforSelectingProposals__c</t>
-  </si>
-  <si>
-    <t>criteria</t>
-  </si>
-  <si>
-    <t>fieldFormulaandMatchingRequirements__c</t>
-  </si>
-  <si>
-    <t>formula</t>
-  </si>
-  <si>
-    <t>fieldLengthandTimePhasingofAssistance__c</t>
-  </si>
-  <si>
-    <t>lengthandtime</t>
-  </si>
-  <si>
-    <t>fieldReports__c</t>
-  </si>
-  <si>
-    <t>reports</t>
-  </si>
-  <si>
-    <t>fieldAudits__c</t>
-  </si>
-  <si>
-    <t>audits</t>
-  </si>
-  <si>
-    <t>fieldRecords__c</t>
-  </si>
-  <si>
-    <t>records</t>
-  </si>
-  <si>
-    <t>fieldRegulationsGuidelinesAndLiterature__c</t>
-  </si>
-  <si>
-    <t>regulations</t>
-  </si>
-  <si>
-    <t>fieldAccountIdentification__c</t>
-  </si>
-  <si>
-    <t>accIdentification</t>
-  </si>
-  <si>
-    <t>fieldObligations__c</t>
-  </si>
-  <si>
-    <t>obligations</t>
-  </si>
-  <si>
-    <t>fieldRangeandAverageofFinancialAssistanc__c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">range </t>
-  </si>
-  <si>
-    <t>fieldProgramAccomplishments__c</t>
-  </si>
-  <si>
-    <t>accomplishments</t>
-  </si>
-  <si>
-    <t>fieldRegionalOrLocalOffice__c</t>
-  </si>
-  <si>
-    <t>rehional</t>
-  </si>
-  <si>
-    <t>fieldHeadquartersOffice__c</t>
-  </si>
-  <si>
-    <t>headq</t>
-  </si>
-  <si>
-    <t>fieldWebsiteAddress__c</t>
-  </si>
-  <si>
-    <t>website</t>
-  </si>
-  <si>
-    <t>fieldMailingCity</t>
-  </si>
-  <si>
-    <t>fieldMailingState</t>
-  </si>
-  <si>
-    <t>fieldNonFederalOrgamizationType__c</t>
-  </si>
-  <si>
-    <t>fieldDUNS__c</t>
-  </si>
-  <si>
-    <t>fieldAuthorizedOrganizationContact__c</t>
-  </si>
-  <si>
-    <t>fieldProjectAbstract__c</t>
-  </si>
-  <si>
-    <t>fieldLocation__c</t>
-  </si>
-  <si>
-    <t>fieldSupplementalFundsRequest__c</t>
-  </si>
-  <si>
-    <t>fieldAre_any_state_specific_forms_attached__c</t>
-  </si>
-  <si>
-    <t>fieldAre_space_requirements_met__c</t>
-  </si>
-  <si>
-    <t>fieldIT_requirements_met__c</t>
-  </si>
-  <si>
-    <t>fieldTraining_Requirements_Met__c</t>
-  </si>
-  <si>
-    <t>fieldAre_special_award_conditions_addressed__c</t>
-  </si>
-  <si>
-    <t>fieldAddition_pending_requirements__c</t>
-  </si>
-  <si>
-    <t>Checklist</t>
-  </si>
-  <si>
-    <t>India</t>
-  </si>
-  <si>
-    <t>Project Abstract Value</t>
-  </si>
-  <si>
-    <t>Automation PM</t>
-  </si>
-  <si>
-    <t>Automation Runtime Contact</t>
-  </si>
-  <si>
-    <t>Automation External Federal Contact</t>
-  </si>
-  <si>
-    <t>Contact</t>
-  </si>
-  <si>
-    <t>Automation Runtime FederalContactsLengthCheck</t>
-  </si>
-  <si>
-    <t>AutomationExernalContactToCheckMaximum0123AutomationExernalContactToCheckMaximum0123</t>
-  </si>
-  <si>
-    <t>Test Address</t>
-  </si>
-  <si>
-    <t>Automation Runtime NF Program</t>
-  </si>
-  <si>
-    <t>Automation Runtime Internal Program</t>
-  </si>
-  <si>
-    <t>Automation Runtime NF Organization</t>
-  </si>
-  <si>
-    <t>No Match</t>
-  </si>
-  <si>
-    <t>Automation Internal Org</t>
-  </si>
-  <si>
-    <t>Automation Runtime Lead</t>
-  </si>
-  <si>
-    <t>aaaaaaaaa</t>
-  </si>
-  <si>
-    <t>fieldLevelofEffort__c</t>
-  </si>
-  <si>
-    <t>aaaaaa</t>
-  </si>
-  <si>
-    <t>aaaaaaa</t>
-  </si>
-  <si>
-    <t>sssssss</t>
-  </si>
-  <si>
-    <t>fieldDetailTechnicalKnowledge__c</t>
-  </si>
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>fieldExplainRequiredResources__c</t>
-  </si>
-  <si>
-    <t>tst</t>
-  </si>
-  <si>
-    <t>fieldExplainRequiredRequirements__c</t>
-  </si>
-  <si>
-    <t>fieldEstimatedFTEToBeHired__c</t>
-  </si>
-  <si>
-    <t>Personnel</t>
+    <t>fieldLaverageAllowed__c</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -710,18 +704,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF222222"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="6"/>
-      <color rgb="FF222222"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -732,19 +714,18 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="5"/>
+      <color rgb="FF333333"/>
+      <name val="Helvetica"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8E8E8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -760,7 +741,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -781,9 +762,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -830,20 +808,17 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1226,7 +1201,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
@@ -1237,7 +1212,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
@@ -1248,7 +1223,7 @@
         <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -1288,21 +1263,21 @@
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="11" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="23" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1344,7 +1319,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="50.4" x14ac:dyDescent="0.3">
@@ -1355,7 +1330,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
@@ -1366,7 +1341,7 @@
         <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
@@ -1412,7 +1387,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D415097A-F360-43DD-83BE-32D88672EF13}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
@@ -1439,7 +1414,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
@@ -1450,34 +1425,45 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="26" customFormat="1" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="s">
+    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+      <c r="A6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" xr:uid="{BAB72A48-CAAE-4FBF-9639-3BA0F69A08EA}"/>
+    <hyperlink ref="C5" r:id="rId1" xr:uid="{BAB72A48-CAAE-4FBF-9639-3BA0F69A08EA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
@@ -1556,8 +1542,8 @@
       <c r="B6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>47</v>
+      <c r="C6" s="35" t="s">
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -1818,7 +1804,7 @@
       <c r="B8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="10" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1842,80 +1828,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="27" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A2" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="29" t="s">
+      <c r="A2" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="29" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+      <c r="A3" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="30" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A3" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="29" t="s">
+      <c r="C3" s="30" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+      <c r="A4" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+      <c r="A5" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="31" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A4" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" s="29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A5" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="29" t="s">
+      <c r="C5" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="32" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+      <c r="A6" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="28" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A6" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="29" t="s">
+      <c r="C6" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="32" t="s">
-        <v>53</v>
-      </c>
     </row>
     <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A7" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="29" t="s">
+      <c r="A7" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="26" t="s">
         <v>56</v>
-      </c>
-      <c r="C7" s="27" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1949,33 +1935,33 @@
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>58</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>60</v>
+      <c r="B3" s="13" t="s">
+        <v>59</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>177</v>
+      <c r="B4" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -2008,55 +1994,55 @@
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>174</v>
+      <c r="B2" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="16" t="s">
         <v>62</v>
-      </c>
-      <c r="C3" s="17" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="16" t="s">
         <v>64</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="14" t="s">
         <v>66</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>68</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2128,7 +2114,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AE13280-37FF-469C-B491-B5A066179CFD}">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" customWidth="1"/>
@@ -2137,333 +2123,278 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" s="37" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
-        <v>55</v>
+      <c r="A2" s="37" t="s">
+        <v>54</v>
       </c>
       <c r="B2" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="33" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="37">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="36" t="s">
         <v>70</v>
       </c>
-      <c r="C2" s="34">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="C3" s="34">
+      <c r="C4" s="37">
         <v>199</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" s="36" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" s="34" t="s">
+    <row r="5" spans="1:3" s="26" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="C5" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" s="26" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>188</v>
+      </c>
+      <c r="C7" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="37" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B5" s="36" t="s">
+      <c r="B8" s="37" t="s">
         <v>74</v>
       </c>
-      <c r="C5" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B6" s="36" t="s">
+      <c r="C8" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="37" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="34" t="s">
+      <c r="C9" s="37" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="34" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="37" t="s">
+        <v>177</v>
+      </c>
+      <c r="C11" s="37" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="33" t="s">
+        <v>179</v>
+      </c>
+      <c r="C13" s="37" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>78</v>
+      </c>
+      <c r="C14" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>181</v>
+      </c>
+      <c r="C15" s="37" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>173</v>
+      </c>
+      <c r="C16" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B17" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="C17" s="34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="C18" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B20" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B21" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B22" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B23" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" s="37" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" s="37" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" s="37" t="s">
         <v>176</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B8" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B9" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="C9" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B10" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="C10" s="34" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B11" s="34" t="s">
-        <v>79</v>
-      </c>
-      <c r="C11" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B12" s="34" t="s">
-        <v>80</v>
-      </c>
-      <c r="C12" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B13" s="34" t="s">
-        <v>81</v>
-      </c>
-      <c r="C13" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B14" s="34" t="s">
-        <v>180</v>
-      </c>
-      <c r="C14" s="34">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B15" s="34" t="s">
-        <v>82</v>
-      </c>
-      <c r="C15" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B16" s="34" t="s">
-        <v>83</v>
-      </c>
-      <c r="C16" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B17" s="34" t="s">
-        <v>84</v>
-      </c>
-      <c r="C17" s="34">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B18" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="C18" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B19" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="C19" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B20" s="34" t="s">
-        <v>87</v>
-      </c>
-      <c r="C20" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B21" s="34" t="s">
-        <v>88</v>
-      </c>
-      <c r="C21" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B22" s="34" t="s">
-        <v>89</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B23" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="C23" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B24" s="34" t="s">
-        <v>91</v>
-      </c>
-      <c r="C24" s="34" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B25" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="C25" s="34" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B26" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="C26" s="34" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B27" s="34" t="s">
-        <v>184</v>
-      </c>
-      <c r="C27" s="34" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B28" s="35" t="s">
-        <v>186</v>
-      </c>
-      <c r="C28" s="34" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B29" s="34" t="s">
-        <v>188</v>
-      </c>
-      <c r="C29" s="34" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B30" s="34" t="s">
-        <v>189</v>
-      </c>
-      <c r="C30" s="33">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2483,344 +2414,344 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="C2" s="21">
+      <c r="A2" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="20">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="20" t="s">
+      <c r="A3" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C4" s="20" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" s="20" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" s="21" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="22" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="20" t="s">
+      <c r="C8" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="C5" s="21" t="s">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="22" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" s="21" t="s">
+      <c r="C9" s="20" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="23" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C10" s="20" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="23" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C11" s="20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="23" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C12" s="20" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="23" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C13" s="20" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="23" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C14" s="20" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" s="23" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="22" t="s">
         <v>109</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C15" s="20" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="23" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="C16" s="20" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" s="23" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C17" s="20" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15" s="23" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="22" t="s">
         <v>115</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C18" s="20" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B16" s="23" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="22" t="s">
         <v>117</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C19" s="20" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B17" s="23" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="C20" s="20" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B18" s="23" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C21" s="20" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B19" s="23" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="C22" s="20" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B20" s="23" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="C20" s="21" t="s">
+      <c r="C23" s="20" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B21" s="23" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="C21" s="21" t="s">
+      <c r="C24" s="20" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B22" s="23" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="C25" s="20" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B23" s="23" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="C23" s="21" t="s">
+      <c r="C26" s="20" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B24" s="23" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="C27" s="20" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B25" s="23" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C28" s="20" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B26" s="23" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="C29" s="20" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B27" s="23" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B30" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="C30" s="20" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B28" s="23" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="C31" s="20" t="s">
         <v>142</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B29" s="23" t="s">
-        <v>143</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B30" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="C30" s="21" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="C31" s="21" t="s">
-        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -3058,7 +2989,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
@@ -3069,7 +3000,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
@@ -3134,7 +3065,7 @@
       <c r="B9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="23" t="s">
         <v>38</v>
       </c>
     </row>
@@ -3142,10 +3073,10 @@
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="C10" s="24" t="s">
+      <c r="B10" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="C10" s="23" t="s">
         <v>39</v>
       </c>
     </row>
@@ -3153,8 +3084,8 @@
       <c r="A11" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="12" t="s">
-        <v>150</v>
+      <c r="B11" s="11" t="s">
+        <v>144</v>
       </c>
       <c r="C11" t="s">
         <v>40</v>
@@ -3179,79 +3110,79 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="37" t="s">
+      <c r="B1" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="37" t="s">
+      <c r="C1" s="32" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="38" t="s">
+      <c r="A2" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="32" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="38" t="s">
+      <c r="A3" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="39">
+      <c r="C3" s="34">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="38" t="s">
+      <c r="A4" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="38" t="s">
-        <v>190</v>
+      <c r="C4" s="33" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="38" t="s">
+      <c r="A5" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="38" t="s">
+      <c r="C5" s="33" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="38" t="s">
+      <c r="A6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="39">
+      <c r="C6" s="34">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="38" t="s">
+      <c r="A7" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="39">
+      <c r="C7" s="34">
         <v>365</v>
       </c>
     </row>
@@ -3282,68 +3213,68 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="38" t="s">
+      <c r="A2" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="32" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="38" t="s">
+      <c r="A3" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="39">
+      <c r="C3" s="34">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="38" t="s">
+      <c r="A4" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="38" t="s">
-        <v>190</v>
+      <c r="C4" s="33" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="38" t="s">
+      <c r="A5" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="38" t="s">
+      <c r="C5" s="33" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="38" t="s">
+      <c r="A6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="39">
+      <c r="C6" s="34">
         <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="38" t="s">
+      <c r="A7" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="39">
+      <c r="C7" s="34">
         <v>365</v>
       </c>
     </row>
@@ -3380,7 +3311,7 @@
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
@@ -3453,11 +3384,11 @@
       <c r="A9" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="25" t="s">
-        <v>151</v>
+      <c r="B9" s="24" t="s">
+        <v>145</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -3480,22 +3411,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="17" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C2">
         <v>456123789</v>
@@ -3503,112 +3434,112 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>153</v>
+        <v>54</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>147</v>
       </c>
       <c r="C3" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C4" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C5" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B6" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B7" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B8" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="C8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B9" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="C9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B10" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B11" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B12" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Grantee changes in Leads Feature...added Activate button click
</commit_message>
<xml_diff>
--- a/src/main/resources/Field_Values.xlsx
+++ b/src/main/resources/Field_Values.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22827"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E681FD-7FD9-426A-8CE6-7BE9E951B5BE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{005C0353-B856-4ABD-A908-F37A23C6C0C0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="16" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="16" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ContactCreation" sheetId="1" r:id="rId1"/>
@@ -741,7 +741,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -819,6 +819,9 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1102,14 +1105,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.21875" customWidth="1"/>
-    <col min="3" max="3" width="31.5546875" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.19921875" customWidth="1"/>
+    <col min="3" max="3" width="31.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1120,7 +1123,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1131,7 +1134,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1142,7 +1145,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1153,7 +1156,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1176,13 +1179,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAD7FB55-E8AD-485D-A372-6318A9353130}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="18.88671875" customWidth="1"/>
-    <col min="3" max="3" width="31.44140625" customWidth="1"/>
+    <col min="2" max="2" width="18.86328125" customWidth="1"/>
+    <col min="3" max="3" width="31.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1193,7 +1196,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1204,7 +1207,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1215,7 +1218,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1226,7 +1229,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1237,7 +1240,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1248,7 +1251,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1259,7 +1262,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1270,7 +1273,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -1293,14 +1296,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E3D1CB4-74AD-4C7B-86A6-6D8597EFB79A}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="43.77734375" customWidth="1"/>
+    <col min="3" max="3" width="43.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1311,7 +1314,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1322,7 +1325,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="49.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1333,7 +1336,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1344,7 +1347,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1355,7 +1358,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1366,7 +1369,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1388,14 +1391,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D415097A-F360-43DD-83BE-32D88672EF13}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.21875" customWidth="1"/>
-    <col min="3" max="3" width="28.21875" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.19921875" customWidth="1"/>
+    <col min="3" max="3" width="28.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1406,7 +1409,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1417,7 +1420,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1428,7 +1431,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="26" customFormat="1" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" s="26" customFormat="1" ht="33" x14ac:dyDescent="0.45">
       <c r="A4" s="27" t="s">
         <v>3</v>
       </c>
@@ -1439,7 +1442,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1450,7 +1453,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1473,14 +1476,14 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C84DBADC-4CFE-43C9-B33B-FB1978F25849}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.77734375" customWidth="1"/>
-    <col min="3" max="3" width="26.88671875" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.796875" customWidth="1"/>
+    <col min="3" max="3" width="26.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1491,7 +1494,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1502,7 +1505,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1513,7 +1516,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1524,7 +1527,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1535,7 +1538,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1558,13 +1561,13 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{410A8461-2BAC-4994-A5A0-900D2EAF4F3E}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="24.109375" customWidth="1"/>
-    <col min="3" max="3" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.1328125" customWidth="1"/>
+    <col min="3" max="3" width="22.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1575,7 +1578,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1586,7 +1589,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1597,7 +1600,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1619,13 +1622,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAFCF55F-195A-445C-9058-59993E2BC9ED}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="27.44140625" customWidth="1"/>
-    <col min="3" max="3" width="26.21875" customWidth="1"/>
+    <col min="2" max="2" width="27.46484375" customWidth="1"/>
+    <col min="3" max="3" width="26.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1636,7 +1639,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1647,7 +1650,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1658,7 +1661,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1669,7 +1672,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1680,7 +1683,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1691,7 +1694,7 @@
         <v>12345678</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1713,14 +1716,14 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDD507A7-A1D7-4C66-91DC-C17845AA6092}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="255.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="255.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1731,7 +1734,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1742,7 +1745,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1753,7 +1756,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1764,7 +1767,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1775,7 +1778,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1786,7 +1789,7 @@
         <v>12345678</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1797,7 +1800,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1820,14 +1823,14 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25B9AAB7-BC0B-48A4-8063-5D4A8BC952DC}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" customWidth="1"/>
-    <col min="2" max="2" width="26.5546875" customWidth="1"/>
-    <col min="3" max="3" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.46484375" customWidth="1"/>
+    <col min="2" max="2" width="26.53125" customWidth="1"/>
+    <col min="3" max="3" width="40.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
@@ -1838,7 +1841,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A2" s="27" t="s">
         <v>3</v>
       </c>
@@ -1849,7 +1852,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A3" s="27" t="s">
         <v>3</v>
       </c>
@@ -1860,18 +1863,18 @@
         <v>171</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A4" s="27" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="C4" s="28">
+      <c r="C4" s="38">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="27" t="s">
         <v>3</v>
       </c>
@@ -1882,7 +1885,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="27" t="s">
         <v>3</v>
       </c>
@@ -1893,7 +1896,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" s="27" t="s">
         <v>3</v>
       </c>
@@ -1913,14 +1916,14 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D57C0A7E-0484-41B3-98B5-765D1318644D}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="19.109375" customWidth="1"/>
-    <col min="2" max="2" width="26.77734375" customWidth="1"/>
+    <col min="1" max="1" width="19.1328125" customWidth="1"/>
+    <col min="2" max="2" width="26.796875" customWidth="1"/>
     <col min="3" max="3" width="42.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1931,7 +1934,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1942,7 +1945,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1953,7 +1956,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1972,14 +1975,14 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90D837CB-E465-4E28-A130-5D8C398A0EED}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="13.6640625" customWidth="1"/>
-    <col min="2" max="2" width="36.5546875" customWidth="1"/>
-    <col min="3" max="3" width="57.88671875" customWidth="1"/>
+    <col min="2" max="2" width="36.53125" customWidth="1"/>
+    <col min="3" max="3" width="57.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1990,7 +1993,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2001,7 +2004,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -2012,7 +2015,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -2023,7 +2026,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2034,7 +2037,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2053,14 +2056,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07A8DFDE-CC9C-46BE-84ED-CACACDED0505}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5546875" customWidth="1"/>
+    <col min="3" max="3" width="23.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2071,7 +2074,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2082,7 +2085,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -2093,7 +2096,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -2115,14 +2118,14 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AE13280-37FF-469C-B491-B5A066179CFD}">
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" customWidth="1"/>
+    <col min="1" max="1" width="12.53125" customWidth="1"/>
     <col min="2" max="2" width="41.6640625" customWidth="1"/>
-    <col min="3" max="3" width="52.5546875" customWidth="1"/>
+    <col min="3" max="3" width="52.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
@@ -2133,7 +2136,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="37" t="s">
         <v>54</v>
       </c>
@@ -2144,7 +2147,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="36" t="s">
         <v>54</v>
       </c>
@@ -2155,7 +2158,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="37" t="s">
         <v>54</v>
       </c>
@@ -2166,7 +2169,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="5" spans="1:3" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" s="26" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A5" s="37" t="s">
         <v>54</v>
       </c>
@@ -2177,7 +2180,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" s="37" t="s">
         <v>54</v>
       </c>
@@ -2188,7 +2191,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:3" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" s="26" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A7" s="37" t="s">
         <v>54</v>
       </c>
@@ -2199,7 +2202,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" s="37" t="s">
         <v>73</v>
       </c>
@@ -2210,7 +2213,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="37" t="s">
         <v>73</v>
       </c>
@@ -2221,7 +2224,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" s="37" t="s">
         <v>73</v>
       </c>
@@ -2232,7 +2235,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" s="37" t="s">
         <v>73</v>
       </c>
@@ -2243,7 +2246,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" s="37" t="s">
         <v>73</v>
       </c>
@@ -2254,7 +2257,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" s="37" t="s">
         <v>73</v>
       </c>
@@ -2265,7 +2268,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" s="37" t="s">
         <v>73</v>
       </c>
@@ -2276,7 +2279,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" s="37" t="s">
         <v>73</v>
       </c>
@@ -2287,7 +2290,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" s="37" t="s">
         <v>73</v>
       </c>
@@ -2298,7 +2301,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" s="37" t="s">
         <v>73</v>
       </c>
@@ -2309,7 +2312,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" s="37" t="s">
         <v>73</v>
       </c>
@@ -2320,7 +2323,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" s="37" t="s">
         <v>73</v>
       </c>
@@ -2331,7 +2334,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" s="37" t="s">
         <v>73</v>
       </c>
@@ -2342,7 +2345,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" s="37" t="s">
         <v>73</v>
       </c>
@@ -2353,7 +2356,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" s="37" t="s">
         <v>73</v>
       </c>
@@ -2364,7 +2367,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" s="37" t="s">
         <v>73</v>
       </c>
@@ -2375,7 +2378,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" s="37" t="s">
         <v>73</v>
       </c>
@@ -2386,7 +2389,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" s="37" t="s">
         <v>73</v>
       </c>
@@ -2406,14 +2409,14 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C9D7AD-DD13-4E10-B333-6FC741B3BFBF}">
   <dimension ref="A1:C31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="11.109375" customWidth="1"/>
-    <col min="2" max="2" width="39.5546875" customWidth="1"/>
+    <col min="1" max="1" width="11.1328125" customWidth="1"/>
+    <col min="2" max="2" width="39.53125" customWidth="1"/>
     <col min="3" max="3" width="40.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
@@ -2424,7 +2427,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="18" t="s">
         <v>3</v>
       </c>
@@ -2435,7 +2438,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="18" t="s">
         <v>3</v>
       </c>
@@ -2446,7 +2449,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="18" t="s">
         <v>3</v>
       </c>
@@ -2457,7 +2460,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" s="18" t="s">
         <v>3</v>
       </c>
@@ -2468,7 +2471,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" s="21" t="s">
         <v>3</v>
       </c>
@@ -2479,7 +2482,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" s="21" t="s">
         <v>3</v>
       </c>
@@ -2490,7 +2493,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" s="21" t="s">
         <v>3</v>
       </c>
@@ -2501,7 +2504,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="21" t="s">
         <v>3</v>
       </c>
@@ -2512,7 +2515,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" s="21" t="s">
         <v>3</v>
       </c>
@@ -2523,7 +2526,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" s="21" t="s">
         <v>3</v>
       </c>
@@ -2534,7 +2537,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" s="21" t="s">
         <v>3</v>
       </c>
@@ -2545,7 +2548,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" s="21" t="s">
         <v>3</v>
       </c>
@@ -2556,7 +2559,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" s="21" t="s">
         <v>3</v>
       </c>
@@ -2567,7 +2570,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" s="21" t="s">
         <v>3</v>
       </c>
@@ -2578,7 +2581,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" s="21" t="s">
         <v>3</v>
       </c>
@@ -2589,7 +2592,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" s="21" t="s">
         <v>3</v>
       </c>
@@ -2600,7 +2603,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" s="21" t="s">
         <v>3</v>
       </c>
@@ -2611,7 +2614,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" s="21" t="s">
         <v>3</v>
       </c>
@@ -2622,7 +2625,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" s="21" t="s">
         <v>3</v>
       </c>
@@ -2633,7 +2636,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" s="21" t="s">
         <v>3</v>
       </c>
@@ -2644,7 +2647,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" s="21" t="s">
         <v>3</v>
       </c>
@@ -2655,7 +2658,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" s="21" t="s">
         <v>3</v>
       </c>
@@ -2666,7 +2669,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" s="21" t="s">
         <v>3</v>
       </c>
@@ -2677,7 +2680,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" s="21" t="s">
         <v>3</v>
       </c>
@@ -2688,7 +2691,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" s="21" t="s">
         <v>3</v>
       </c>
@@ -2699,7 +2702,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A27" s="21" t="s">
         <v>3</v>
       </c>
@@ -2710,7 +2713,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A28" s="21" t="s">
         <v>3</v>
       </c>
@@ -2721,7 +2724,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A29" s="21" t="s">
         <v>3</v>
       </c>
@@ -2732,7 +2735,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A30" s="21" t="s">
         <v>3</v>
       </c>
@@ -2743,7 +2746,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A31" s="21" t="s">
         <v>3</v>
       </c>
@@ -2762,14 +2765,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C825052-5BFB-48CE-AF18-A05985C2E861}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" customWidth="1"/>
-    <col min="3" max="3" width="26.21875" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.46484375" customWidth="1"/>
+    <col min="3" max="3" width="26.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2780,7 +2783,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2791,7 +2794,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -2802,7 +2805,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -2813,7 +2816,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2824,7 +2827,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -2835,7 +2838,7 @@
         <v>12345678</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -2857,14 +2860,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C54FC4-ECE0-4935-82B1-FA8D76408EA8}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="2" width="23.44140625" customWidth="1"/>
-    <col min="3" max="3" width="30.88671875" customWidth="1"/>
+    <col min="1" max="1" width="14.796875" customWidth="1"/>
+    <col min="2" max="2" width="23.46484375" customWidth="1"/>
+    <col min="3" max="3" width="30.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2875,7 +2878,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2886,7 +2889,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -2897,7 +2900,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -2908,7 +2911,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2919,7 +2922,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -2930,7 +2933,7 @@
         <v>12345678</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -2941,7 +2944,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -2963,14 +2966,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E468D78-1254-4AD2-810C-41AE4E131ED6}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" customWidth="1"/>
-    <col min="2" max="2" width="25.5546875" customWidth="1"/>
+    <col min="1" max="1" width="18.46484375" customWidth="1"/>
+    <col min="2" max="2" width="25.53125" customWidth="1"/>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2981,7 +2984,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2992,7 +2995,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -3003,7 +3006,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -3014,7 +3017,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -3025,7 +3028,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -3036,7 +3039,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -3047,7 +3050,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -3058,7 +3061,7 @@
         <v>41102</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -3069,7 +3072,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -3080,7 +3083,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>3</v>
       </c>
@@ -3103,13 +3106,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3165D747-C28E-4C3E-96DA-2777CB00933A}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="25.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
@@ -3120,7 +3123,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="32" t="s">
         <v>3</v>
       </c>
@@ -3131,7 +3134,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="32" t="s">
         <v>3</v>
       </c>
@@ -3142,7 +3145,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="32" t="s">
         <v>3</v>
       </c>
@@ -3153,7 +3156,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" s="32" t="s">
         <v>3</v>
       </c>
@@ -3164,7 +3167,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" s="32" t="s">
         <v>3</v>
       </c>
@@ -3175,7 +3178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" s="32" t="s">
         <v>3</v>
       </c>
@@ -3195,13 +3198,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE2AE6E5-9BA0-4079-BFA8-85F960DC3870}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="25.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3212,7 +3215,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="32" t="s">
         <v>3</v>
       </c>
@@ -3223,7 +3226,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="32" t="s">
         <v>3</v>
       </c>
@@ -3234,7 +3237,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="32" t="s">
         <v>3</v>
       </c>
@@ -3245,7 +3248,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" s="32" t="s">
         <v>3</v>
       </c>
@@ -3256,7 +3259,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" s="32" t="s">
         <v>3</v>
       </c>
@@ -3267,7 +3270,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" s="32" t="s">
         <v>3</v>
       </c>
@@ -3286,13 +3289,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB063D14-2E1A-4894-A22D-BD2B91269468}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="25.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.19921875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3303,7 +3306,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3314,7 +3317,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3325,7 +3328,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3336,7 +3339,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -3347,7 +3350,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -3358,7 +3361,7 @@
         <v>20301</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -3369,7 +3372,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -3380,7 +3383,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -3403,14 +3406,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A2F5532-64E8-4157-849F-E59312F5A712}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="44.21875" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" customWidth="1"/>
+    <col min="2" max="2" width="44.19921875" customWidth="1"/>
+    <col min="3" max="3" width="20.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -3421,7 +3424,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>54</v>
       </c>
@@ -3432,7 +3435,7 @@
         <v>456123789</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>54</v>
       </c>
@@ -3443,7 +3446,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>54</v>
       </c>
@@ -3454,7 +3457,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>54</v>
       </c>
@@ -3465,7 +3468,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>54</v>
       </c>
@@ -3476,7 +3479,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>157</v>
       </c>
@@ -3487,7 +3490,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>157</v>
       </c>
@@ -3498,7 +3501,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>157</v>
       </c>
@@ -3509,7 +3512,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>157</v>
       </c>
@@ -3520,7 +3523,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>157</v>
       </c>
@@ -3531,7 +3534,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>157</v>
       </c>

</xml_diff>

<commit_message>
1.Completed 5 test cases on 2 july with earlier completed scenarios 2. Refactored stuff for Grantee
</commit_message>
<xml_diff>
--- a/src/main/resources/Field_Values.xlsx
+++ b/src/main/resources/Field_Values.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22827"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{005C0353-B856-4ABD-A908-F37A23C6C0C0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{831E3C88-4380-4EBE-88B6-CA7DF4F9FBEC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="16" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="18" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ContactCreation" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,8 @@
     <sheet name="ProgramsExternalNFProgram" sheetId="17" r:id="rId18"/>
     <sheet name="ProgramsInternalProgram" sheetId="18" r:id="rId19"/>
     <sheet name="OpportunityDetails" sheetId="19" r:id="rId20"/>
-    <sheet name="EditNonFederalProgram" sheetId="20" r:id="rId21"/>
+    <sheet name="OpportunityDetailsWithPreApp" sheetId="25" r:id="rId21"/>
+    <sheet name="EditNonFederalProgram" sheetId="20" r:id="rId22"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="190">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -607,6 +608,9 @@
   </si>
   <si>
     <t>fieldLaverageAllowed__c</t>
+  </si>
+  <si>
+    <t>fieldPreApplicationNeeded__c</t>
   </si>
 </sst>
 </file>
@@ -2407,6 +2411,308 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44B94B75-16C2-45C8-8C5C-21179AF7DBFC}">
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.59765625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="33" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="37">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="37">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="C5" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>188</v>
+      </c>
+      <c r="C7" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" s="26" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="C8" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="37" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" s="37" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="37" t="s">
+        <v>177</v>
+      </c>
+      <c r="C12" s="37" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A13" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A14" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>179</v>
+      </c>
+      <c r="C14" s="37" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A15" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>78</v>
+      </c>
+      <c r="C15" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A16" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>181</v>
+      </c>
+      <c r="C16" s="37" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A17" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B17" s="37" t="s">
+        <v>173</v>
+      </c>
+      <c r="C17" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A18" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="C18" s="34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A19" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A20" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B20" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A21" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B21" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="C21" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A22" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B22" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="C22" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A23" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B23" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23" s="37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A24" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="C24" s="37" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A25" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="C25" s="37" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A26" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B26" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="C26" s="37" t="s">
+        <v>176</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C9D7AD-DD13-4E10-B333-6FC741B3BFBF}">
   <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>

</xml_diff>

<commit_message>
1.Completed 6 scenarios 2. Refactored Grantee Home and planning stuff
</commit_message>
<xml_diff>
--- a/src/main/resources/Field_Values.xlsx
+++ b/src/main/resources/Field_Values.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22827"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{831E3C88-4380-4EBE-88B6-CA7DF4F9FBEC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4BF48E2-A786-4A8C-8CCE-01B076742787}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="18" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ContactCreation" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
1.Completed 5 scenarios 2. Modified Leads feature for grantee
</commit_message>
<xml_diff>
--- a/src/main/resources/Field_Values.xlsx
+++ b/src/main/resources/Field_Values.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22827"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4BF48E2-A786-4A8C-8CCE-01B076742787}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47490303-3850-456D-9CC5-21926BC7D35C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="14" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ContactCreation" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
updated opportunity - pre application
</commit_message>
<xml_diff>
--- a/src/main/resources/Field_Values.xlsx
+++ b/src/main/resources/Field_Values.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23001"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47490303-3850-456D-9CC5-21926BC7D35C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F709FC70-1FB8-42D0-9C4E-B669EA685EF0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="14" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="16" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ContactCreation" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="192">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -611,6 +611,12 @@
   </si>
   <si>
     <t>fieldPreApplicationNeeded__c</t>
+  </si>
+  <si>
+    <t>fieldLeadAgencyAgreedUpon__c</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -2121,7 +2127,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AE13280-37FF-469C-B491-B5A066179CFD}">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12.53125" customWidth="1"/>
@@ -2338,15 +2344,15 @@
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:3" s="26" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A20" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="B20" s="37" t="s">
-        <v>81</v>
+      <c r="B20" s="11" t="s">
+        <v>190</v>
       </c>
       <c r="C20" s="37" t="s">
-        <v>56</v>
+        <v>191</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.45">
@@ -2354,7 +2360,7 @@
         <v>73</v>
       </c>
       <c r="B21" s="37" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C21" s="37" t="s">
         <v>56</v>
@@ -2365,7 +2371,7 @@
         <v>73</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C22" s="37" t="s">
         <v>56</v>
@@ -2376,10 +2382,10 @@
         <v>73</v>
       </c>
       <c r="B23" s="37" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C23" s="37" t="s">
-        <v>174</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.45">
@@ -2387,10 +2393,10 @@
         <v>73</v>
       </c>
       <c r="B24" s="37" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C24" s="37" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.45">
@@ -2398,9 +2404,20 @@
         <v>73</v>
       </c>
       <c r="B25" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="C25" s="37" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A26" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B26" s="37" t="s">
         <v>87</v>
       </c>
-      <c r="C25" s="37" t="s">
+      <c r="C26" s="37" t="s">
         <v>176</v>
       </c>
     </row>

</xml_diff>

<commit_message>
!.Refactord Grantee organization, kpi, strategic  plan, focus area 2. Refactored HOme module
</commit_message>
<xml_diff>
--- a/src/main/resources/Field_Values.xlsx
+++ b/src/main/resources/Field_Values.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23001"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F709FC70-1FB8-42D0-9C4E-B669EA685EF0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D8D72B-3BF6-4ECB-A1F9-457F78B5E59A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="16" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ContactCreation" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="193">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -145,9 +145,6 @@
     <t>fieldBillingCity</t>
   </si>
   <si>
-    <t>fieldBillingState</t>
-  </si>
-  <si>
     <t>fieldBillingPostalCode</t>
   </si>
   <si>
@@ -478,9 +475,6 @@
     <t>fieldMailingState</t>
   </si>
   <si>
-    <t>fieldNonFederalOrgamizationType__c</t>
-  </si>
-  <si>
     <t>fieldDUNS__c</t>
   </si>
   <si>
@@ -617,6 +611,15 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>fieldNonFederalOrganizationType__c</t>
+  </si>
+  <si>
+    <t>fieldState__c</t>
+  </si>
+  <si>
+    <t>ARNFO</t>
   </si>
 </sst>
 </file>
@@ -1214,7 +1217,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
@@ -1225,7 +1228,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="33" x14ac:dyDescent="0.45">
@@ -1236,7 +1239,7 @@
         <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
@@ -1247,7 +1250,7 @@
         <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -1266,10 +1269,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>44</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
@@ -1280,7 +1283,7 @@
         <v>18</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
@@ -1332,7 +1335,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="49.5" x14ac:dyDescent="0.45">
@@ -1343,7 +1346,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
@@ -1354,7 +1357,7 @@
         <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
@@ -1365,7 +1368,7 @@
         <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -1384,10 +1387,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>44</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1427,7 +1430,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
@@ -1438,7 +1441,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="26" customFormat="1" ht="33" x14ac:dyDescent="0.45">
@@ -1449,7 +1452,7 @@
         <v>21</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
@@ -1460,7 +1463,7 @@
         <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -1534,7 +1537,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -1553,10 +1556,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -1856,10 +1859,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C2" s="29" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -1867,10 +1870,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C3" s="30" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -1878,7 +1881,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C4" s="38">
         <v>0</v>
@@ -1889,10 +1892,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="31" t="s">
         <v>49</v>
-      </c>
-      <c r="C5" s="31" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -1900,10 +1903,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="31" t="s">
         <v>51</v>
-      </c>
-      <c r="C6" s="31" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -1911,10 +1914,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="26" t="s">
         <v>55</v>
-      </c>
-      <c r="C7" s="26" t="s">
-        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1949,10 +1952,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>57</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -1960,10 +1963,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -1971,10 +1974,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -2008,10 +2011,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
@@ -2019,10 +2022,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="16" t="s">
         <v>61</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
@@ -2030,10 +2033,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="16" t="s">
         <v>63</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
@@ -2041,10 +2044,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="14" t="s">
         <v>65</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
@@ -2052,10 +2055,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>67</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -2148,21 +2151,21 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="33" t="s">
         <v>71</v>
-      </c>
-      <c r="C2" s="33" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="36" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" s="36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C3" s="37">
         <v>49</v>
@@ -2170,10 +2173,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" s="36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C4" s="37">
         <v>199</v>
@@ -2181,131 +2184,131 @@
     </row>
     <row r="5" spans="1:3" s="26" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A5" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="26" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A7" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="37" t="s">
-        <v>74</v>
-      </c>
       <c r="C8" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C13" s="37" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C15" s="37" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C16" s="37">
         <v>3</v>
@@ -2313,10 +2316,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C17" s="34">
         <v>2</v>
@@ -2324,101 +2327,101 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C18" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C19" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:3" s="26" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A20" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C20" s="37" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B21" s="37" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C21" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C22" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B23" s="37" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C23" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B24" s="37" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C24" s="37" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B25" s="37" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C25" s="37" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B26" s="37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C26" s="37" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2450,21 +2453,21 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="33" t="s">
         <v>71</v>
-      </c>
-      <c r="C2" s="33" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="36" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" s="36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C3" s="37">
         <v>49</v>
@@ -2472,10 +2475,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" s="36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C4" s="37">
         <v>199</v>
@@ -2483,142 +2486,142 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="26" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A8" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="B9" s="37" t="s">
-        <v>74</v>
-      </c>
       <c r="C9" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C13" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C15" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C16" s="37" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C17" s="37">
         <v>3</v>
@@ -2626,10 +2629,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C18" s="34">
         <v>2</v>
@@ -2637,90 +2640,90 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C19" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B20" s="37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C20" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B21" s="37" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C21" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C22" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B23" s="37" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C23" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B24" s="37" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C24" s="37" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B25" s="37" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C25" s="37" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B26" s="37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C26" s="37" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2755,7 +2758,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C2" s="20">
         <v>3</v>
@@ -2766,10 +2769,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
@@ -2777,10 +2780,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
@@ -2788,10 +2791,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="C5" s="20" t="s">
         <v>90</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
@@ -2799,10 +2802,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
@@ -2810,10 +2813,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" s="20" t="s">
         <v>93</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -2821,10 +2824,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="C8" s="20" t="s">
         <v>95</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
@@ -2832,10 +2835,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="C9" s="20" t="s">
         <v>97</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
@@ -2843,10 +2846,10 @@
         <v>3</v>
       </c>
       <c r="B10" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" s="20" t="s">
         <v>99</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.45">
@@ -2854,10 +2857,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="C11" s="20" t="s">
         <v>101</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
@@ -2865,10 +2868,10 @@
         <v>3</v>
       </c>
       <c r="B12" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="C12" s="20" t="s">
         <v>103</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.45">
@@ -2876,10 +2879,10 @@
         <v>3</v>
       </c>
       <c r="B13" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="C13" s="20" t="s">
         <v>105</v>
-      </c>
-      <c r="C13" s="20" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.45">
@@ -2887,10 +2890,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" s="20" t="s">
         <v>107</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.45">
@@ -2898,10 +2901,10 @@
         <v>3</v>
       </c>
       <c r="B15" s="22" t="s">
+        <v>108</v>
+      </c>
+      <c r="C15" s="20" t="s">
         <v>109</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.45">
@@ -2909,10 +2912,10 @@
         <v>3</v>
       </c>
       <c r="B16" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="C16" s="20" t="s">
         <v>111</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.45">
@@ -2920,10 +2923,10 @@
         <v>3</v>
       </c>
       <c r="B17" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C17" s="20" t="s">
         <v>113</v>
-      </c>
-      <c r="C17" s="20" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.45">
@@ -2931,10 +2934,10 @@
         <v>3</v>
       </c>
       <c r="B18" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="C18" s="20" t="s">
         <v>115</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.45">
@@ -2942,10 +2945,10 @@
         <v>3</v>
       </c>
       <c r="B19" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="C19" s="20" t="s">
         <v>117</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.45">
@@ -2953,10 +2956,10 @@
         <v>3</v>
       </c>
       <c r="B20" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C20" s="20" t="s">
         <v>119</v>
-      </c>
-      <c r="C20" s="20" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.45">
@@ -2964,10 +2967,10 @@
         <v>3</v>
       </c>
       <c r="B21" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="C21" s="20" t="s">
         <v>121</v>
-      </c>
-      <c r="C21" s="20" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.45">
@@ -2975,10 +2978,10 @@
         <v>3</v>
       </c>
       <c r="B22" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="C22" s="20" t="s">
         <v>123</v>
-      </c>
-      <c r="C22" s="20" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.45">
@@ -2986,10 +2989,10 @@
         <v>3</v>
       </c>
       <c r="B23" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="C23" s="20" t="s">
         <v>125</v>
-      </c>
-      <c r="C23" s="20" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.45">
@@ -2997,10 +3000,10 @@
         <v>3</v>
       </c>
       <c r="B24" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="C24" s="20" t="s">
         <v>127</v>
-      </c>
-      <c r="C24" s="20" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.45">
@@ -3008,10 +3011,10 @@
         <v>3</v>
       </c>
       <c r="B25" s="22" t="s">
+        <v>128</v>
+      </c>
+      <c r="C25" s="20" t="s">
         <v>129</v>
-      </c>
-      <c r="C25" s="20" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.45">
@@ -3019,10 +3022,10 @@
         <v>3</v>
       </c>
       <c r="B26" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="C26" s="20" t="s">
         <v>131</v>
-      </c>
-      <c r="C26" s="20" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.45">
@@ -3030,10 +3033,10 @@
         <v>3</v>
       </c>
       <c r="B27" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="C27" s="20" t="s">
         <v>133</v>
-      </c>
-      <c r="C27" s="20" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.45">
@@ -3041,10 +3044,10 @@
         <v>3</v>
       </c>
       <c r="B28" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="C28" s="20" t="s">
         <v>135</v>
-      </c>
-      <c r="C28" s="20" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.45">
@@ -3052,10 +3055,10 @@
         <v>3</v>
       </c>
       <c r="B29" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="C29" s="20" t="s">
         <v>137</v>
-      </c>
-      <c r="C29" s="20" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.45">
@@ -3063,10 +3066,10 @@
         <v>3</v>
       </c>
       <c r="B30" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="C30" s="20" t="s">
         <v>139</v>
-      </c>
-      <c r="C30" s="20" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.45">
@@ -3074,10 +3077,10 @@
         <v>3</v>
       </c>
       <c r="B31" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="C31" s="20" t="s">
         <v>141</v>
-      </c>
-      <c r="C31" s="20" t="s">
-        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -3315,7 +3318,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
@@ -3326,7 +3329,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
@@ -3392,7 +3395,7 @@
         <v>18</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
@@ -3400,10 +3403,10 @@
         <v>3</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
@@ -3411,10 +3414,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -3476,7 +3479,7 @@
         <v>29</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
@@ -3568,7 +3571,7 @@
         <v>29</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
@@ -3611,7 +3614,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB063D14-2E1A-4894-A22D-BD2B91269468}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="25.19921875" bestFit="1" customWidth="1"/>
@@ -3637,7 +3640,7 @@
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -3648,7 +3651,7 @@
         <v>32</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -3659,18 +3662,18 @@
         <v>33</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>34</v>
+      <c r="B5" s="11" t="s">
+        <v>191</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -3678,7 +3681,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6" s="8">
         <v>20301</v>
@@ -3689,10 +3692,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
@@ -3700,21 +3703,32 @@
         <v>3</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A9" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="24" t="s">
-        <v>145</v>
+      <c r="B9" s="11" t="s">
+        <v>190</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A10" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -3749,10 +3763,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C2">
         <v>456123789</v>
@@ -3760,112 +3774,112 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C5" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B9" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B11" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>